<commit_message>
fix(sprint2): align test plan with 24 types §4.12, clean SRS-1.1, and sync defect register
</commit_message>
<xml_diff>
--- a/docs/sprint2/requirements-defects.xlsx
+++ b/docs/sprint2/requirements-defects.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Реєстр" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Розподіл розділів" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Спірні" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="5 питань замовника" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Аудит_Бучинський" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Аудит_Панайотов" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Аудит_Костенко" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Аудит_Пархоменко" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Аудит_Кираківський" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Статистика" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реєстр" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Розподіл розділів" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Спірні" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 питань замовника" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудит_Бучинський" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудит_Панайотов" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудит_Костенко" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудит_Пархоменко" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудит_Кираківський" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Статистика" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -654,7 +654,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Кираківський О., 5ani0chek</t>
+          <t>Панайотов О., Кираківський О.</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Бучинський Д., Vov4ik</t>
+          <t>Бучинський Д., Костенко В.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Кираківський О., Бучинський Д.</t>
+          <t>Кираківський О.</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Vov4ik, Пархоменко О.</t>
+          <t>Костенко В.</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>5ani0chek, Бучинський Д.</t>
+          <t>Панайотов О.</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Бучинський Д., Vov4ik</t>
+          <t>Бучинський Д., Костенко В.</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Бучинський Д., Кираківський О.</t>
+          <t>Бучинський Д., Панайотов О., Кираківський О.</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Бучинський Д., Vov4ik</t>
+          <t>Бучинський Д., Костенко В.</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>5ani0chek, Пархоменко О.</t>
+          <t>Панайотов О., Пархоменко О.</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Пархоменко О., Кираківський О.</t>
+          <t>Пархоменко О.</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Бучинський Д., 5ani0chek</t>
+          <t>Бучинський Д., Панайотов О.</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Бучинський Д., Vov4ik</t>
+          <t>Бучинський Д., Костенко В.</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Кираківський О., Бучинський Д.</t>
+          <t>Кираківський О.</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Пархоменко О., Vov4ik</t>
+          <t>Пархоменко О.</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Кираківський О., Бучинський Д.</t>
+          <t>Кираківський О.</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Бучинський Д., 5ani0chek</t>
+          <t>Бучинський Д., Панайотов О.</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Vov4ik, Бучинський Д.</t>
+          <t>Костенко В.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Бучинський Д., Vov4ik</t>
+          <t>Бучинський Д., Костенко В.</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Кираківський О., Пархоменко О.</t>
+          <t>Пархоменко О.</t>
         </is>
       </c>
     </row>
@@ -1673,11 +1673,11 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>29.17%</t>
+          <t>37.50%</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1693,11 +1693,11 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>25.00%</t>
+          <t>29.17%</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1713,16 +1713,16 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>20.83%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>BL-20, BL-50, BL-80 (+ перехресні F-60/BL-30)</t>
+          <t>BL-20, BL-50, BL-80</t>
         </is>
       </c>
     </row>
@@ -1733,16 +1733,16 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>25.00%</t>
+          <t>20.83%</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>D-10, P-20, D-20, U-20, U-10 (+ перехресні F-10/S-20)</t>
+          <t>D-10, P-20, D-20, U-20, U-10</t>
         </is>
       </c>
     </row>

</xml_diff>